<commit_message>
Sync armor workbook and CE patch values
</commit_message>
<xml_diff>
--- a/RimWorld CE Ayameduki Race Patching and Stats - reviewed.xlsx
+++ b/RimWorld CE Ayameduki Race Patching and Stats - reviewed.xlsx
@@ -1641,7 +1641,7 @@
       </c>
       <c r="C11" s="106" t="inlineStr">
         <is>
-          <t>HAR_NM_sh_BKo</t>
+          <t>HAR_NM_Sh_BKo</t>
         </is>
       </c>
       <c r="D11" s="107" t="inlineStr">
@@ -1661,7 +1661,9 @@
         </is>
       </c>
       <c r="H11" s="104" t="inlineStr"/>
-      <c r="I11" s="117" t="inlineStr"/>
+      <c r="I11" s="117" t="n">
+        <v>1</v>
+      </c>
       <c r="J11" s="117" t="inlineStr"/>
       <c r="K11" s="117" t="inlineStr"/>
       <c r="L11" s="116" t="n">
@@ -1976,12 +1978,12 @@
       </c>
       <c r="F16" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G16" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H16" s="104" t="inlineStr">
@@ -1989,7 +1991,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I16" s="117" t="inlineStr"/>
+      <c r="I16" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J16" s="116" t="n">
         <v>0.3</v>
       </c>
@@ -1999,7 +2003,9 @@
       <c r="L16" s="116" t="n">
         <v>0.3</v>
       </c>
-      <c r="M16" s="119" t="inlineStr"/>
+      <c r="M16" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N16" s="118" t="n">
         <v>4</v>
       </c>
@@ -2050,12 +2056,12 @@
       </c>
       <c r="F17" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G17" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H17" s="104" t="inlineStr">
@@ -2063,7 +2069,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I17" s="117" t="inlineStr"/>
+      <c r="I17" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J17" s="116" t="n">
         <v>0.3</v>
       </c>
@@ -2073,7 +2081,9 @@
       <c r="L17" s="116" t="n">
         <v>0.3</v>
       </c>
-      <c r="M17" s="119" t="inlineStr"/>
+      <c r="M17" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N17" s="118" t="n">
         <v>4</v>
       </c>
@@ -2190,12 +2200,12 @@
       </c>
       <c r="F19" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G19" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H19" s="104" t="inlineStr">
@@ -2203,7 +2213,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I19" s="117" t="inlineStr"/>
+      <c r="I19" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J19" s="116" t="n">
         <v>0.3</v>
       </c>
@@ -2213,7 +2225,9 @@
       <c r="L19" s="116" t="n">
         <v>0.3</v>
       </c>
-      <c r="M19" s="119" t="inlineStr"/>
+      <c r="M19" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N19" s="118" t="n">
         <v>4</v>
       </c>
@@ -2264,7 +2278,7 @@
       </c>
       <c r="F20" s="113" t="inlineStr">
         <is>
-          <t>CE Carry Weight, CE Bulk Capacity</t>
+          <t>CE Carry Weight, CE Bulk Capacity, CE Material</t>
         </is>
       </c>
       <c r="G20" s="113" t="inlineStr">
@@ -2277,7 +2291,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I20" s="117" t="inlineStr"/>
+      <c r="I20" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J20" s="116" t="n">
         <v>1.2</v>
       </c>
@@ -2287,7 +2303,9 @@
       <c r="L20" s="116" t="n">
         <v>1.2</v>
       </c>
-      <c r="M20" s="119" t="inlineStr"/>
+      <c r="M20" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N20" s="118" t="n">
         <v>12</v>
       </c>
@@ -2342,12 +2360,12 @@
       </c>
       <c r="F21" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G21" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H21" s="104" t="inlineStr">
@@ -2355,7 +2373,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I21" s="117" t="inlineStr"/>
+      <c r="I21" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J21" s="116" t="n">
         <v>1.2</v>
       </c>
@@ -2365,7 +2385,9 @@
       <c r="L21" s="116" t="n">
         <v>1.2</v>
       </c>
-      <c r="M21" s="119" t="inlineStr"/>
+      <c r="M21" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N21" s="118" t="n">
         <v>12</v>
       </c>
@@ -2420,12 +2442,12 @@
       </c>
       <c r="F22" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G22" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H22" s="104" t="inlineStr">
@@ -2433,7 +2455,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I22" s="117" t="inlineStr"/>
+      <c r="I22" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J22" s="116" t="n">
         <v>1.2</v>
       </c>
@@ -2443,7 +2467,9 @@
       <c r="L22" s="116" t="n">
         <v>1.2</v>
       </c>
-      <c r="M22" s="119" t="inlineStr"/>
+      <c r="M22" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N22" s="118" t="n">
         <v>12</v>
       </c>
@@ -2498,7 +2524,7 @@
       </c>
       <c r="F23" s="113" t="inlineStr">
         <is>
-          <t>CE Night Vision</t>
+          <t>CE Night Vision, CE Material</t>
         </is>
       </c>
       <c r="G23" s="113" t="inlineStr">
@@ -2511,7 +2537,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I23" s="117" t="inlineStr"/>
+      <c r="I23" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J23" s="116" t="n">
         <v>0.5</v>
       </c>
@@ -2521,7 +2549,9 @@
       <c r="L23" s="116" t="n">
         <v>0.5</v>
       </c>
-      <c r="M23" s="119" t="inlineStr"/>
+      <c r="M23" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N23" s="118" t="n">
         <v>8</v>
       </c>
@@ -2849,7 +2879,7 @@
       </c>
       <c r="C29" s="106" t="inlineStr">
         <is>
-          <t>HAR_NM_SH_Kc</t>
+          <t>HAR_NM_Sh_Kc</t>
         </is>
       </c>
       <c r="D29" s="107" t="inlineStr">
@@ -4694,7 +4724,7 @@
       </c>
       <c r="F60" s="113" t="inlineStr">
         <is>
-          <t>CE Carry Weight, CE Bulk Capacity</t>
+          <t>CE Carry Weight, CE Bulk Capacity, CE Material</t>
         </is>
       </c>
       <c r="G60" s="113" t="inlineStr">
@@ -4707,7 +4737,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I60" s="117" t="inlineStr"/>
+      <c r="I60" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J60" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -4717,7 +4749,9 @@
       <c r="L60" s="116" t="n">
         <v>1.5</v>
       </c>
-      <c r="M60" s="119" t="inlineStr"/>
+      <c r="M60" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N60" s="118" t="n">
         <v>22</v>
       </c>
@@ -4772,7 +4806,7 @@
       </c>
       <c r="F61" s="113" t="inlineStr">
         <is>
-          <t>CE Night Vision</t>
+          <t>CE Night Vision, CE Material</t>
         </is>
       </c>
       <c r="G61" s="113" t="inlineStr">
@@ -4785,7 +4819,9 @@
           <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
         </is>
       </c>
-      <c r="I61" s="117" t="inlineStr"/>
+      <c r="I61" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J61" s="116" t="n">
         <v>1.6</v>
       </c>
@@ -4795,7 +4831,9 @@
       <c r="L61" s="116" t="n">
         <v>1.6</v>
       </c>
-      <c r="M61" s="119" t="inlineStr"/>
+      <c r="M61" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N61" s="118" t="n">
         <v>18</v>
       </c>
@@ -4963,17 +5001,27 @@
       </c>
       <c r="E64" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F64" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F64" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Sharp, CE Blunt, CE Heat, CE Bulk, CE Worn Bulk</t>
+        </is>
+      </c>
       <c r="G64" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H64" s="104" t="inlineStr"/>
-      <c r="I64" s="117" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H64" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Nearmare/ThingDefs_Misc/Nearmare_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I64" s="117" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J64" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -4983,7 +5031,9 @@
       <c r="L64" s="116" t="n">
         <v>1.5</v>
       </c>
-      <c r="M64" s="119" t="inlineStr"/>
+      <c r="M64" s="119" t="n">
+        <v>0.5</v>
+      </c>
       <c r="N64" s="118" t="n">
         <v>16</v>
       </c>
@@ -5034,12 +5084,12 @@
       </c>
       <c r="F65" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material, CE Heat</t>
         </is>
       </c>
       <c r="G65" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H65" s="104" t="inlineStr">
@@ -5047,7 +5097,9 @@
           <t>Patches/Littluna/ThingDefs_Misc/Littluna_Apparel.xml</t>
         </is>
       </c>
-      <c r="I65" s="117" t="inlineStr"/>
+      <c r="I65" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J65" s="116" t="n">
         <v>1.3</v>
       </c>
@@ -5057,14 +5109,18 @@
       <c r="L65" s="116" t="n">
         <v>1.3</v>
       </c>
-      <c r="M65" s="119" t="inlineStr"/>
+      <c r="M65" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N65" s="118" t="n">
         <v>20</v>
       </c>
       <c r="O65" s="118" t="n">
         <v>44</v>
       </c>
-      <c r="P65" s="119" t="inlineStr"/>
+      <c r="P65" s="119" t="n">
+        <v>1.3</v>
+      </c>
       <c r="Q65" s="118" t="n">
         <v>80</v>
       </c>
@@ -5110,12 +5166,12 @@
       </c>
       <c r="F66" s="104" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt, CE Material, CE Heat</t>
         </is>
       </c>
       <c r="G66" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H66" s="104" t="inlineStr">
@@ -5123,7 +5179,9 @@
           <t>Patches/Littluna/ThingDefs_Misc/Littluna_Apparel.xml</t>
         </is>
       </c>
-      <c r="I66" s="117" t="inlineStr"/>
+      <c r="I66" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J66" s="116" t="n">
         <v>1.3</v>
       </c>
@@ -5133,14 +5191,18 @@
       <c r="L66" s="116" t="n">
         <v>1.3</v>
       </c>
-      <c r="M66" s="119" t="inlineStr"/>
+      <c r="M66" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N66" s="118" t="n">
         <v>18</v>
       </c>
       <c r="O66" s="118" t="n">
         <v>38</v>
       </c>
-      <c r="P66" s="119" t="inlineStr"/>
+      <c r="P66" s="119" t="n">
+        <v>1.3</v>
+      </c>
       <c r="Q66" s="118" t="n">
         <v>40</v>
       </c>
@@ -5934,12 +5996,12 @@
       </c>
       <c r="F80" s="104" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G80" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H80" s="104" t="inlineStr">
@@ -5947,7 +6009,9 @@
           <t>Patches/Idearn Race/ThingDefs_Misc/Idearn_Apparel.xml</t>
         </is>
       </c>
-      <c r="I80" s="117" t="inlineStr"/>
+      <c r="I80" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J80" s="116" t="n">
         <v>1</v>
       </c>
@@ -5957,7 +6021,9 @@
       <c r="L80" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M80" s="119" t="inlineStr"/>
+      <c r="M80" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N80" s="118" t="n">
         <v>16</v>
       </c>
@@ -6012,12 +6078,12 @@
       </c>
       <c r="F81" s="104" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G81" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H81" s="104" t="inlineStr">
@@ -6025,7 +6091,9 @@
           <t>Patches/Idearn Race/ThingDefs_Misc/Idearn_Apparel.xml</t>
         </is>
       </c>
-      <c r="I81" s="117" t="inlineStr"/>
+      <c r="I81" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J81" s="116" t="n">
         <v>1</v>
       </c>
@@ -6035,7 +6103,9 @@
       <c r="L81" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M81" s="119" t="inlineStr"/>
+      <c r="M81" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N81" s="118" t="n">
         <v>14</v>
       </c>
@@ -6088,12 +6158,12 @@
       </c>
       <c r="F82" s="104" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G82" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H82" s="104" t="inlineStr">
@@ -6101,7 +6171,9 @@
           <t>Patches/Idearn Race/ThingDefs_Misc/Idearn_Apparel.xml</t>
         </is>
       </c>
-      <c r="I82" s="117" t="inlineStr"/>
+      <c r="I82" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J82" s="116" t="n">
         <v>2</v>
       </c>
@@ -6111,7 +6183,9 @@
       <c r="L82" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M82" s="119" t="inlineStr"/>
+      <c r="M82" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N82" s="118" t="n">
         <v>28</v>
       </c>
@@ -6386,12 +6460,12 @@
       </c>
       <c r="F86" s="104" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G86" s="109" t="inlineStr">
         <is>
-          <t>Matches repo patch</t>
+          <t>Updated to match repo patch</t>
         </is>
       </c>
       <c r="H86" s="104" t="inlineStr">
@@ -6399,7 +6473,9 @@
           <t>Patches/Idearn Race/ThingDefs_Misc/Idearn_Apparel.xml</t>
         </is>
       </c>
-      <c r="I86" s="117" t="inlineStr"/>
+      <c r="I86" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J86" s="116" t="n">
         <v>2</v>
       </c>
@@ -6409,7 +6485,9 @@
       <c r="L86" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M86" s="119" t="inlineStr"/>
+      <c r="M86" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N86" s="118" t="n">
         <v>24</v>
       </c>
@@ -6936,7 +7014,7 @@
       </c>
       <c r="F95" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
         </is>
       </c>
       <c r="G95" s="113" t="inlineStr">
@@ -6954,13 +7032,17 @@
       </c>
       <c r="J95" s="117" t="inlineStr"/>
       <c r="K95" s="117" t="inlineStr"/>
-      <c r="L95" s="117" t="inlineStr"/>
+      <c r="L95" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M95" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N95" s="119" t="inlineStr"/>
       <c r="O95" s="119" t="inlineStr"/>
-      <c r="P95" s="119" t="inlineStr"/>
+      <c r="P95" s="119" t="n">
+        <v>2</v>
+      </c>
       <c r="Q95" s="118" t="n">
         <v>1</v>
       </c>
@@ -7002,7 +7084,7 @@
       </c>
       <c r="F96" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
         </is>
       </c>
       <c r="G96" s="113" t="inlineStr">
@@ -7020,13 +7102,17 @@
       </c>
       <c r="J96" s="117" t="inlineStr"/>
       <c r="K96" s="117" t="inlineStr"/>
-      <c r="L96" s="117" t="inlineStr"/>
+      <c r="L96" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M96" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N96" s="119" t="inlineStr"/>
       <c r="O96" s="119" t="inlineStr"/>
-      <c r="P96" s="119" t="inlineStr"/>
+      <c r="P96" s="119" t="n">
+        <v>2</v>
+      </c>
       <c r="Q96" s="118" t="n">
         <v>1</v>
       </c>
@@ -7068,7 +7154,7 @@
       </c>
       <c r="F97" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
         </is>
       </c>
       <c r="G97" s="113" t="inlineStr">
@@ -7086,13 +7172,17 @@
       </c>
       <c r="J97" s="117" t="inlineStr"/>
       <c r="K97" s="117" t="inlineStr"/>
-      <c r="L97" s="117" t="inlineStr"/>
+      <c r="L97" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M97" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N97" s="119" t="inlineStr"/>
       <c r="O97" s="119" t="inlineStr"/>
-      <c r="P97" s="119" t="inlineStr"/>
+      <c r="P97" s="119" t="n">
+        <v>2</v>
+      </c>
       <c r="Q97" s="118" t="n">
         <v>1</v>
       </c>
@@ -7134,7 +7224,7 @@
       </c>
       <c r="F98" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
         </is>
       </c>
       <c r="G98" s="113" t="inlineStr">
@@ -7152,13 +7242,17 @@
       </c>
       <c r="J98" s="117" t="inlineStr"/>
       <c r="K98" s="117" t="inlineStr"/>
-      <c r="L98" s="117" t="inlineStr"/>
+      <c r="L98" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M98" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N98" s="119" t="inlineStr"/>
       <c r="O98" s="119" t="inlineStr"/>
-      <c r="P98" s="119" t="inlineStr"/>
+      <c r="P98" s="119" t="n">
+        <v>2</v>
+      </c>
       <c r="Q98" s="118" t="n">
         <v>10</v>
       </c>
@@ -7185,7 +7279,7 @@
       </c>
       <c r="C99" s="106" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_c</t>
+          <t>HAR_CO_Apparel_Head_c</t>
         </is>
       </c>
       <c r="D99" s="108" t="inlineStr">
@@ -7195,30 +7289,46 @@
       </c>
       <c r="E99" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F99" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F99" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
+        </is>
+      </c>
       <c r="G99" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H99" s="104" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H99" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
+        </is>
+      </c>
       <c r="I99" s="116" t="n">
         <v>0</v>
       </c>
       <c r="J99" s="117" t="inlineStr"/>
       <c r="K99" s="117" t="inlineStr"/>
-      <c r="L99" s="117" t="inlineStr"/>
+      <c r="L99" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M99" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N99" s="119" t="inlineStr"/>
       <c r="O99" s="119" t="inlineStr"/>
-      <c r="P99" s="119" t="inlineStr"/>
-      <c r="Q99" s="119" t="inlineStr"/>
-      <c r="R99" s="119" t="inlineStr"/>
+      <c r="P99" s="119" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q99" s="119" t="n">
+        <v>1</v>
+      </c>
+      <c r="R99" s="119" t="n">
+        <v>1</v>
+      </c>
       <c r="S99" s="119" t="inlineStr"/>
       <c r="T99" s="119" t="inlineStr"/>
       <c r="U99" s="119" t="inlineStr"/>
@@ -7239,7 +7349,7 @@
       </c>
       <c r="C100" s="106" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_b</t>
+          <t>HAR_CO_Apparel_Head_b</t>
         </is>
       </c>
       <c r="D100" s="108" t="inlineStr">
@@ -7249,30 +7359,46 @@
       </c>
       <c r="E100" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F100" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F100" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
+        </is>
+      </c>
       <c r="G100" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H100" s="104" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H100" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
+        </is>
+      </c>
       <c r="I100" s="116" t="n">
         <v>0</v>
       </c>
       <c r="J100" s="117" t="inlineStr"/>
       <c r="K100" s="117" t="inlineStr"/>
-      <c r="L100" s="117" t="inlineStr"/>
+      <c r="L100" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M100" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N100" s="119" t="inlineStr"/>
       <c r="O100" s="119" t="inlineStr"/>
-      <c r="P100" s="119" t="inlineStr"/>
-      <c r="Q100" s="119" t="inlineStr"/>
-      <c r="R100" s="119" t="inlineStr"/>
+      <c r="P100" s="119" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q100" s="119" t="n">
+        <v>1</v>
+      </c>
+      <c r="R100" s="119" t="n">
+        <v>1</v>
+      </c>
       <c r="S100" s="119" t="inlineStr"/>
       <c r="T100" s="119" t="inlineStr"/>
       <c r="U100" s="119" t="inlineStr"/>
@@ -7293,7 +7419,7 @@
       </c>
       <c r="C101" s="106" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_a</t>
+          <t>HAR_CO_Apparel_Head_a</t>
         </is>
       </c>
       <c r="D101" s="108" t="inlineStr">
@@ -7303,30 +7429,46 @@
       </c>
       <c r="E101" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F101" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F101" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Heat</t>
+        </is>
+      </c>
       <c r="G101" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H101" s="104" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H101" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
+        </is>
+      </c>
       <c r="I101" s="116" t="n">
         <v>0</v>
       </c>
       <c r="J101" s="117" t="inlineStr"/>
       <c r="K101" s="117" t="inlineStr"/>
-      <c r="L101" s="117" t="inlineStr"/>
+      <c r="L101" s="117" t="n">
+        <v>2</v>
+      </c>
       <c r="M101" s="118" t="n">
         <v>0</v>
       </c>
       <c r="N101" s="119" t="inlineStr"/>
       <c r="O101" s="119" t="inlineStr"/>
-      <c r="P101" s="119" t="inlineStr"/>
-      <c r="Q101" s="119" t="inlineStr"/>
-      <c r="R101" s="119" t="inlineStr"/>
+      <c r="P101" s="119" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q101" s="119" t="n">
+        <v>1</v>
+      </c>
+      <c r="R101" s="119" t="n">
+        <v>1</v>
+      </c>
       <c r="S101" s="119" t="inlineStr"/>
       <c r="T101" s="119" t="inlineStr"/>
       <c r="U101" s="119" t="inlineStr"/>
@@ -7335,186 +7477,72 @@
       </c>
     </row>
     <row r="102" ht="12" customHeight="1" s="49">
-      <c r="A102" s="104" t="inlineStr">
-        <is>
-          <t>Chaoura</t>
-        </is>
-      </c>
-      <c r="B102" s="105" t="inlineStr">
-        <is>
-          <t>[missing from original sheet]</t>
-        </is>
-      </c>
-      <c r="C102" s="106" t="inlineStr">
-        <is>
-          <t>HAR_CO_Apparel_Head_a</t>
-        </is>
-      </c>
-      <c r="D102" s="108" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E102" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F102" s="104" t="inlineStr">
-        <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
-        </is>
-      </c>
-      <c r="G102" s="114" t="inlineStr">
-        <is>
-          <t>Missing from original workbook</t>
-        </is>
-      </c>
-      <c r="H102" s="114" t="inlineStr">
-        <is>
-          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
-        </is>
-      </c>
+      <c r="A102" s="104" t="n"/>
+      <c r="B102" s="105" t="n"/>
+      <c r="C102" s="106" t="n"/>
+      <c r="D102" s="108" t="n"/>
+      <c r="E102" s="112" t="n"/>
+      <c r="F102" s="104" t="n"/>
+      <c r="G102" s="114" t="n"/>
+      <c r="H102" s="114" t="n"/>
       <c r="I102" s="117" t="inlineStr"/>
       <c r="J102" s="117" t="inlineStr"/>
       <c r="K102" s="117" t="inlineStr"/>
       <c r="L102" s="117" t="inlineStr"/>
-      <c r="M102" s="118" t="n">
-        <v>0</v>
-      </c>
+      <c r="M102" s="118" t="n"/>
       <c r="N102" s="119" t="inlineStr"/>
       <c r="O102" s="119" t="inlineStr"/>
       <c r="P102" s="119" t="inlineStr"/>
-      <c r="Q102" s="118" t="n">
-        <v>1</v>
-      </c>
-      <c r="R102" s="118" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q102" s="118" t="n"/>
+      <c r="R102" s="118" t="n"/>
       <c r="S102" s="119" t="inlineStr"/>
       <c r="T102" s="119" t="inlineStr"/>
       <c r="U102" s="119" t="inlineStr"/>
       <c r="V102" s="111" t="inlineStr"/>
     </row>
     <row r="103" ht="12" customHeight="1" s="49">
-      <c r="A103" s="104" t="inlineStr">
-        <is>
-          <t>Chaoura</t>
-        </is>
-      </c>
-      <c r="B103" s="105" t="inlineStr">
-        <is>
-          <t>[missing from original sheet]</t>
-        </is>
-      </c>
-      <c r="C103" s="106" t="inlineStr">
-        <is>
-          <t>HAR_CO_Apparel_Head_b</t>
-        </is>
-      </c>
-      <c r="D103" s="108" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E103" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F103" s="104" t="inlineStr">
-        <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
-        </is>
-      </c>
-      <c r="G103" s="114" t="inlineStr">
-        <is>
-          <t>Missing from original workbook</t>
-        </is>
-      </c>
-      <c r="H103" s="114" t="inlineStr">
-        <is>
-          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
-        </is>
-      </c>
+      <c r="A103" s="104" t="n"/>
+      <c r="B103" s="105" t="n"/>
+      <c r="C103" s="106" t="n"/>
+      <c r="D103" s="108" t="n"/>
+      <c r="E103" s="112" t="n"/>
+      <c r="F103" s="104" t="n"/>
+      <c r="G103" s="114" t="n"/>
+      <c r="H103" s="114" t="n"/>
       <c r="I103" s="117" t="inlineStr"/>
       <c r="J103" s="117" t="inlineStr"/>
       <c r="K103" s="117" t="inlineStr"/>
       <c r="L103" s="117" t="inlineStr"/>
-      <c r="M103" s="118" t="n">
-        <v>0</v>
-      </c>
+      <c r="M103" s="118" t="n"/>
       <c r="N103" s="119" t="inlineStr"/>
       <c r="O103" s="119" t="inlineStr"/>
       <c r="P103" s="119" t="inlineStr"/>
-      <c r="Q103" s="118" t="n">
-        <v>1</v>
-      </c>
-      <c r="R103" s="118" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q103" s="118" t="n"/>
+      <c r="R103" s="118" t="n"/>
       <c r="S103" s="119" t="inlineStr"/>
       <c r="T103" s="119" t="inlineStr"/>
       <c r="U103" s="119" t="inlineStr"/>
       <c r="V103" s="111" t="inlineStr"/>
     </row>
     <row r="104" ht="12" customHeight="1" s="49">
-      <c r="A104" s="104" t="inlineStr">
-        <is>
-          <t>Chaoura</t>
-        </is>
-      </c>
-      <c r="B104" s="105" t="inlineStr">
-        <is>
-          <t>[missing from original sheet]</t>
-        </is>
-      </c>
-      <c r="C104" s="106" t="inlineStr">
-        <is>
-          <t>HAR_CO_Apparel_Head_c</t>
-        </is>
-      </c>
-      <c r="D104" s="108" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E104" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F104" s="104" t="inlineStr">
-        <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk</t>
-        </is>
-      </c>
-      <c r="G104" s="114" t="inlineStr">
-        <is>
-          <t>Missing from original workbook</t>
-        </is>
-      </c>
-      <c r="H104" s="114" t="inlineStr">
-        <is>
-          <t>Patches/Chaoura Race/ThingDefs_Misc/Chaoura_Apparel.xml</t>
-        </is>
-      </c>
+      <c r="A104" s="104" t="n"/>
+      <c r="B104" s="105" t="n"/>
+      <c r="C104" s="106" t="n"/>
+      <c r="D104" s="108" t="n"/>
+      <c r="E104" s="112" t="n"/>
+      <c r="F104" s="104" t="n"/>
+      <c r="G104" s="114" t="n"/>
+      <c r="H104" s="114" t="n"/>
       <c r="I104" s="117" t="inlineStr"/>
       <c r="J104" s="117" t="inlineStr"/>
       <c r="K104" s="117" t="inlineStr"/>
       <c r="L104" s="117" t="inlineStr"/>
-      <c r="M104" s="118" t="n">
-        <v>0</v>
-      </c>
+      <c r="M104" s="118" t="n"/>
       <c r="N104" s="119" t="inlineStr"/>
       <c r="O104" s="119" t="inlineStr"/>
       <c r="P104" s="119" t="inlineStr"/>
-      <c r="Q104" s="118" t="n">
-        <v>1</v>
-      </c>
-      <c r="R104" s="118" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q104" s="118" t="n"/>
+      <c r="R104" s="118" t="n"/>
       <c r="S104" s="119" t="inlineStr"/>
       <c r="T104" s="119" t="inlineStr"/>
       <c r="U104" s="119" t="inlineStr"/>
@@ -8680,7 +8708,7 @@
       </c>
       <c r="F123" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G123" s="113" t="inlineStr">
@@ -8693,7 +8721,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I123" s="117" t="inlineStr"/>
+      <c r="I123" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J123" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -8703,7 +8733,9 @@
       <c r="L123" s="116" t="n">
         <v>1.5</v>
       </c>
-      <c r="M123" s="119" t="inlineStr"/>
+      <c r="M123" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N123" s="118" t="n">
         <v>24</v>
       </c>
@@ -8758,7 +8790,7 @@
       </c>
       <c r="F124" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G124" s="113" t="inlineStr">
@@ -8771,7 +8803,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I124" s="117" t="inlineStr"/>
+      <c r="I124" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J124" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -8781,7 +8815,9 @@
       <c r="L124" s="116" t="n">
         <v>1.5</v>
       </c>
-      <c r="M124" s="119" t="inlineStr"/>
+      <c r="M124" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N124" s="118" t="n">
         <v>24</v>
       </c>
@@ -8819,7 +8855,7 @@
       </c>
       <c r="C125" s="106" t="inlineStr">
         <is>
-          <t>HAR_QA_S_a</t>
+          <t>HAR_QL_S_a</t>
         </is>
       </c>
       <c r="D125" s="108" t="inlineStr">
@@ -8829,17 +8865,27 @@
       </c>
       <c r="E125" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F125" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F125" s="104" t="inlineStr">
+        <is>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material, CE Heat</t>
+        </is>
+      </c>
       <c r="G125" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H125" s="104" t="inlineStr"/>
-      <c r="I125" s="117" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H125" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I125" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J125" s="116" t="n">
         <v>0.5</v>
       </c>
@@ -8849,12 +8895,24 @@
       <c r="L125" s="116" t="n">
         <v>0.5</v>
       </c>
-      <c r="M125" s="119" t="inlineStr"/>
-      <c r="N125" s="119" t="inlineStr"/>
-      <c r="O125" s="119" t="inlineStr"/>
-      <c r="P125" s="119" t="inlineStr"/>
-      <c r="Q125" s="119" t="inlineStr"/>
-      <c r="R125" s="119" t="inlineStr"/>
+      <c r="M125" s="119" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N125" s="119" t="n">
+        <v>5</v>
+      </c>
+      <c r="O125" s="119" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="P125" s="119" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q125" s="119" t="n">
+        <v>40</v>
+      </c>
+      <c r="R125" s="119" t="n">
+        <v>10</v>
+      </c>
       <c r="S125" s="119" t="inlineStr"/>
       <c r="T125" s="119" t="inlineStr"/>
       <c r="U125" s="119" t="inlineStr"/>
@@ -8958,7 +9016,7 @@
       </c>
       <c r="F127" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material, CE Heat</t>
         </is>
       </c>
       <c r="G127" s="113" t="inlineStr">
@@ -8971,7 +9029,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I127" s="117" t="inlineStr"/>
+      <c r="I127" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J127" s="116" t="n">
         <v>0.9</v>
       </c>
@@ -8981,14 +9041,18 @@
       <c r="L127" s="116" t="n">
         <v>0.9</v>
       </c>
-      <c r="M127" s="119" t="inlineStr"/>
+      <c r="M127" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N127" s="118" t="n">
         <v>1</v>
       </c>
       <c r="O127" s="118" t="n">
         <v>1.5</v>
       </c>
-      <c r="P127" s="119" t="inlineStr"/>
+      <c r="P127" s="119" t="n">
+        <v>0.9</v>
+      </c>
       <c r="Q127" s="118" t="n">
         <v>40</v>
       </c>
@@ -9030,7 +9094,7 @@
       </c>
       <c r="F128" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material, CE Heat</t>
         </is>
       </c>
       <c r="G128" s="113" t="inlineStr">
@@ -9043,7 +9107,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I128" s="117" t="inlineStr"/>
+      <c r="I128" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J128" s="116" t="n">
         <v>0.5</v>
       </c>
@@ -9053,14 +9119,18 @@
       <c r="L128" s="116" t="n">
         <v>0.5</v>
       </c>
-      <c r="M128" s="119" t="inlineStr"/>
+      <c r="M128" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N128" s="118" t="n">
         <v>5</v>
       </c>
       <c r="O128" s="118" t="n">
         <v>7.5</v>
       </c>
-      <c r="P128" s="119" t="inlineStr"/>
+      <c r="P128" s="119" t="n">
+        <v>0.5</v>
+      </c>
       <c r="Q128" s="118" t="n">
         <v>40</v>
       </c>
@@ -9102,7 +9172,7 @@
       </c>
       <c r="F129" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt, CE Heat</t>
         </is>
       </c>
       <c r="G129" s="113" t="inlineStr">
@@ -9115,7 +9185,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I129" s="117" t="inlineStr"/>
+      <c r="I129" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J129" s="116" t="n">
         <v>0.4</v>
       </c>
@@ -9134,7 +9206,9 @@
       <c r="O129" s="118" t="n">
         <v>12</v>
       </c>
-      <c r="P129" s="119" t="inlineStr"/>
+      <c r="P129" s="119" t="n">
+        <v>0.4</v>
+      </c>
       <c r="Q129" s="118" t="n">
         <v>0.5</v>
       </c>
@@ -9176,7 +9250,7 @@
       </c>
       <c r="F130" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt, CE Heat</t>
         </is>
       </c>
       <c r="G130" s="113" t="inlineStr">
@@ -9189,7 +9263,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I130" s="117" t="inlineStr"/>
+      <c r="I130" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J130" s="116" t="n">
         <v>0.4</v>
       </c>
@@ -9208,7 +9284,9 @@
       <c r="O130" s="118" t="n">
         <v>12</v>
       </c>
-      <c r="P130" s="119" t="inlineStr"/>
+      <c r="P130" s="119" t="n">
+        <v>0.4</v>
+      </c>
       <c r="Q130" s="118" t="n">
         <v>0.5</v>
       </c>
@@ -9250,7 +9328,7 @@
       </c>
       <c r="F131" s="113" t="inlineStr">
         <is>
-          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt</t>
+          <t>CE Material, CE Bulk, CE Worn Bulk, CE Sharp, CE Blunt, CE Heat</t>
         </is>
       </c>
       <c r="G131" s="113" t="inlineStr">
@@ -9263,7 +9341,9 @@
           <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
         </is>
       </c>
-      <c r="I131" s="117" t="inlineStr"/>
+      <c r="I131" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J131" s="116" t="n">
         <v>0.4</v>
       </c>
@@ -9282,7 +9362,9 @@
       <c r="O131" s="118" t="n">
         <v>12</v>
       </c>
-      <c r="P131" s="119" t="inlineStr"/>
+      <c r="P131" s="119" t="n">
+        <v>0.4</v>
+      </c>
       <c r="Q131" s="118" t="n">
         <v>0.5</v>
       </c>
@@ -9365,64 +9447,24 @@
       </c>
     </row>
     <row r="133" ht="12" customHeight="1" s="49">
-      <c r="A133" s="104" t="inlineStr">
-        <is>
-          <t>Qualeela</t>
-        </is>
-      </c>
-      <c r="B133" s="105" t="inlineStr">
-        <is>
-          <t>[missing from original sheet]</t>
-        </is>
-      </c>
-      <c r="C133" s="106" t="inlineStr">
-        <is>
-          <t>HAR_QL_S_a</t>
-        </is>
-      </c>
-      <c r="D133" s="108" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E133" s="112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F133" s="104" t="inlineStr">
-        <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
-        </is>
-      </c>
-      <c r="G133" s="114" t="inlineStr">
-        <is>
-          <t>Missing from original workbook</t>
-        </is>
-      </c>
-      <c r="H133" s="114" t="inlineStr">
-        <is>
-          <t>Patches/Qualeela Race/ThingDefs_Misc/Qualeela_Apparel.xml</t>
-        </is>
-      </c>
+      <c r="A133" s="104" t="n"/>
+      <c r="B133" s="105" t="n"/>
+      <c r="C133" s="106" t="n"/>
+      <c r="D133" s="108" t="n"/>
+      <c r="E133" s="112" t="n"/>
+      <c r="F133" s="104" t="n"/>
+      <c r="G133" s="114" t="n"/>
+      <c r="H133" s="114" t="n"/>
       <c r="I133" s="117" t="inlineStr"/>
       <c r="J133" s="117" t="inlineStr"/>
       <c r="K133" s="117" t="inlineStr"/>
       <c r="L133" s="117" t="inlineStr"/>
       <c r="M133" s="119" t="inlineStr"/>
-      <c r="N133" s="118" t="n">
-        <v>5</v>
-      </c>
-      <c r="O133" s="118" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="N133" s="118" t="n"/>
+      <c r="O133" s="118" t="n"/>
       <c r="P133" s="119" t="inlineStr"/>
-      <c r="Q133" s="118" t="n">
-        <v>40</v>
-      </c>
-      <c r="R133" s="118" t="n">
-        <v>10</v>
-      </c>
+      <c r="Q133" s="118" t="n"/>
+      <c r="R133" s="118" t="n"/>
       <c r="S133" s="119" t="inlineStr"/>
       <c r="T133" s="119" t="inlineStr"/>
       <c r="U133" s="119" t="inlineStr"/>
@@ -11385,17 +11427,27 @@
       </c>
       <c r="E166" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F166" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F166" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Sharp, CE Blunt, CE Heat, CE Bulk, CE Worn Bulk</t>
+        </is>
+      </c>
       <c r="G166" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H166" s="104" t="inlineStr"/>
-      <c r="I166" s="117" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H166" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Solark Race/ThingDefs_Misc/Solark_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I166" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J166" s="116" t="n">
         <v>0.9</v>
       </c>
@@ -11405,7 +11457,9 @@
       <c r="L166" s="116" t="n">
         <v>0.2</v>
       </c>
-      <c r="M166" s="119" t="inlineStr"/>
+      <c r="M166" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N166" s="118" t="n">
         <v>16</v>
       </c>
@@ -11456,7 +11510,7 @@
       </c>
       <c r="F167" s="113" t="inlineStr">
         <is>
-          <t>CE Night Vision</t>
+          <t>CE Night Vision, CE Material</t>
         </is>
       </c>
       <c r="G167" s="113" t="inlineStr">
@@ -11469,7 +11523,9 @@
           <t>Patches/Solark Race/ThingDefs_Misc/Solark_Apparel.xml</t>
         </is>
       </c>
-      <c r="I167" s="117" t="inlineStr"/>
+      <c r="I167" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J167" s="116" t="n">
         <v>0.9</v>
       </c>
@@ -11479,7 +11535,9 @@
       <c r="L167" s="116" t="n">
         <v>0.1</v>
       </c>
-      <c r="M167" s="119" t="inlineStr"/>
+      <c r="M167" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N167" s="118" t="n">
         <v>18</v>
       </c>
@@ -11585,17 +11643,27 @@
       </c>
       <c r="E169" s="108" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F169" s="104" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F169" s="104" t="inlineStr">
+        <is>
+          <t>CE Material, CE Sharp, CE Blunt</t>
+        </is>
+      </c>
       <c r="G169" s="109" t="inlineStr">
         <is>
-          <t>No current repo patch for this item</t>
-        </is>
-      </c>
-      <c r="H169" s="104" t="inlineStr"/>
-      <c r="I169" s="117" t="inlineStr"/>
+          <t>Updated to match repo patch</t>
+        </is>
+      </c>
+      <c r="H169" s="104" t="inlineStr">
+        <is>
+          <t>Patches/Solark Race/ThingDefs_Misc/Solark_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I169" s="117" t="n">
+        <v>1</v>
+      </c>
       <c r="J169" s="116" t="n">
         <v>0.4</v>
       </c>
@@ -11605,7 +11673,9 @@
       <c r="L169" s="116" t="n">
         <v>0</v>
       </c>
-      <c r="M169" s="119" t="inlineStr"/>
+      <c r="M169" s="119" t="n">
+        <v>1</v>
+      </c>
       <c r="N169" s="118" t="n">
         <v>10</v>
       </c>
@@ -13512,7 +13582,7 @@
       </c>
       <c r="F200" s="113" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G200" s="113" t="inlineStr">
@@ -13525,7 +13595,9 @@
           <t>Patches/Eveliet Race/ThingDefs_Misc/Eveliet_Apparel.xml</t>
         </is>
       </c>
-      <c r="I200" s="117" t="inlineStr"/>
+      <c r="I200" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J200" s="116" t="n">
         <v>1</v>
       </c>
@@ -13535,7 +13607,9 @@
       <c r="L200" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M200" s="119" t="inlineStr"/>
+      <c r="M200" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N200" s="118" t="n">
         <v>18</v>
       </c>
@@ -13590,7 +13664,7 @@
       </c>
       <c r="F201" s="113" t="inlineStr">
         <is>
-          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt</t>
+          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G201" s="113" t="inlineStr">
@@ -13603,7 +13677,9 @@
           <t>Patches/Eveliet Race/ThingDefs_Misc/Eveliet_Apparel.xml</t>
         </is>
       </c>
-      <c r="I201" s="117" t="inlineStr"/>
+      <c r="I201" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J201" s="116" t="n">
         <v>1</v>
       </c>
@@ -13613,7 +13689,9 @@
       <c r="L201" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M201" s="119" t="inlineStr"/>
+      <c r="M201" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N201" s="118" t="n">
         <v>16</v>
       </c>
@@ -15572,7 +15650,7 @@
       </c>
       <c r="F233" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G233" s="113" t="inlineStr">
@@ -15585,7 +15663,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I233" s="117" t="inlineStr"/>
+      <c r="I233" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J233" s="116" t="n">
         <v>1</v>
       </c>
@@ -15595,7 +15675,9 @@
       <c r="L233" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M233" s="119" t="inlineStr"/>
+      <c r="M233" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N233" s="118" t="n">
         <v>18</v>
       </c>
@@ -15648,7 +15730,7 @@
       </c>
       <c r="F234" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Night Vision, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G234" s="113" t="inlineStr">
@@ -15661,7 +15743,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I234" s="117" t="inlineStr"/>
+      <c r="I234" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J234" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -15671,7 +15755,9 @@
       <c r="L234" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M234" s="119" t="inlineStr"/>
+      <c r="M234" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N234" s="118" t="n">
         <v>24</v>
       </c>
@@ -15988,7 +16074,7 @@
       </c>
       <c r="F239" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G239" s="113" t="inlineStr">
@@ -16001,7 +16087,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I239" s="117" t="inlineStr"/>
+      <c r="I239" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J239" s="116" t="n">
         <v>1</v>
       </c>
@@ -16011,7 +16099,9 @@
       <c r="L239" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M239" s="119" t="inlineStr"/>
+      <c r="M239" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N239" s="118" t="n">
         <v>18</v>
       </c>
@@ -16062,7 +16152,7 @@
       </c>
       <c r="F240" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G240" s="113" t="inlineStr">
@@ -16075,7 +16165,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I240" s="117" t="inlineStr"/>
+      <c r="I240" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J240" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -16085,7 +16177,9 @@
       <c r="L240" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M240" s="119" t="inlineStr"/>
+      <c r="M240" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N240" s="118" t="n">
         <v>24</v>
       </c>
@@ -16334,7 +16428,7 @@
       </c>
       <c r="F244" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G244" s="113" t="inlineStr">
@@ -16347,7 +16441,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I244" s="117" t="inlineStr"/>
+      <c r="I244" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J244" s="116" t="n">
         <v>1</v>
       </c>
@@ -16357,7 +16453,9 @@
       <c r="L244" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M244" s="119" t="inlineStr"/>
+      <c r="M244" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N244" s="118" t="n">
         <v>18</v>
       </c>
@@ -16412,7 +16510,7 @@
       </c>
       <c r="F245" s="113" t="inlineStr">
         <is>
-          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt</t>
+          <t>CE Sharp, CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Blunt, CE Material</t>
         </is>
       </c>
       <c r="G245" s="113" t="inlineStr">
@@ -16425,7 +16523,9 @@
           <t>Patches/Zoichor/ThingDefs_Misc/Zoichor_Apparel.xml</t>
         </is>
       </c>
-      <c r="I245" s="117" t="inlineStr"/>
+      <c r="I245" s="117" t="n">
+        <v>0.1</v>
+      </c>
       <c r="J245" s="116" t="n">
         <v>1.5</v>
       </c>
@@ -16435,7 +16535,9 @@
       <c r="L245" s="116" t="n">
         <v>2</v>
       </c>
-      <c r="M245" s="119" t="inlineStr"/>
+      <c r="M245" s="119" t="n">
+        <v>0.1</v>
+      </c>
       <c r="N245" s="118" t="n">
         <v>24</v>
       </c>
@@ -17512,10 +17614,12 @@
       </c>
       <c r="C16" s="70" t="inlineStr">
         <is>
-          <t>HAR_NM_sh_BKo</t>
-        </is>
-      </c>
-      <c r="D16" s="32" t="n"/>
+          <t>HAR_NM_Sh_BKo</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="E16" s="32" t="n"/>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="29" t="n">
@@ -17751,7 +17855,9 @@
           <t>HAR_NM_Sh_Cry</t>
         </is>
       </c>
-      <c r="D21" s="40" t="n"/>
+      <c r="D21" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E21" s="28" t="n">
         <v>0.3</v>
       </c>
@@ -17767,7 +17873,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J21" s="39" t="n"/>
+      <c r="J21" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K21" s="76" t="n">
         <v>4</v>
       </c>
@@ -17799,7 +17907,9 @@
           <t>HAR_NM_AH_h</t>
         </is>
       </c>
-      <c r="D22" s="40" t="n"/>
+      <c r="D22" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E22" s="28" t="n">
         <v>0.3</v>
       </c>
@@ -17815,7 +17925,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J22" s="39" t="n"/>
+      <c r="J22" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K22" s="76" t="n">
         <v>4</v>
       </c>
@@ -17887,7 +17999,9 @@
           <t>HAR_NM_Wear_y</t>
         </is>
       </c>
-      <c r="D24" s="40" t="n"/>
+      <c r="D24" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E24" s="28" t="n">
         <v>0.3</v>
       </c>
@@ -17903,7 +18017,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J24" s="39" t="n"/>
+      <c r="J24" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K24" s="76" t="n">
         <v>4</v>
       </c>
@@ -17935,7 +18051,9 @@
           <t>HAR_NM_A_b</t>
         </is>
       </c>
-      <c r="D25" s="40" t="n"/>
+      <c r="D25" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E25" s="28" t="n">
         <v>1.2</v>
       </c>
@@ -17955,7 +18073,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J25" s="39" t="n"/>
+      <c r="J25" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K25" s="8" t="n">
         <v>12</v>
       </c>
@@ -17991,7 +18111,9 @@
           <t>HAR_NM_A_c</t>
         </is>
       </c>
-      <c r="D26" s="40" t="n"/>
+      <c r="D26" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E26" s="28" t="n">
         <v>1.2</v>
       </c>
@@ -18007,7 +18129,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J26" s="39" t="n"/>
+      <c r="J26" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K26" s="76" t="n">
         <v>12</v>
       </c>
@@ -18043,7 +18167,9 @@
           <t>HAR_NM_A_d</t>
         </is>
       </c>
-      <c r="D27" s="40" t="n"/>
+      <c r="D27" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E27" s="28" t="n">
         <v>1.2</v>
       </c>
@@ -18059,7 +18185,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J27" s="39" t="n"/>
+      <c r="J27" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K27" s="76" t="n">
         <v>12</v>
       </c>
@@ -18095,7 +18223,9 @@
           <t>HAR_NM_AH_g</t>
         </is>
       </c>
-      <c r="D28" s="40" t="n"/>
+      <c r="D28" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E28" s="28" t="n">
         <v>0.5</v>
       </c>
@@ -18115,7 +18245,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J28" s="39" t="n"/>
+      <c r="J28" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K28" s="8" t="n">
         <v>8</v>
       </c>
@@ -18346,7 +18478,7 @@
       </c>
       <c r="C34" s="70" t="inlineStr">
         <is>
-          <t>HAR_NM_SH_Kc</t>
+          <t>HAR_NM_Sh_Kc</t>
         </is>
       </c>
       <c r="D34" s="32" t="n">
@@ -19589,7 +19721,9 @@
           <t>HAR_NM_A_a</t>
         </is>
       </c>
-      <c r="D65" s="41" t="n"/>
+      <c r="D65" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E65" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -19609,7 +19743,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J65" s="39" t="n"/>
+      <c r="J65" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K65" s="8" t="n">
         <v>22</v>
       </c>
@@ -19645,7 +19781,9 @@
           <t>HAR_NM_AH_f</t>
         </is>
       </c>
-      <c r="D66" s="41" t="n"/>
+      <c r="D66" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E66" s="28" t="n">
         <v>1.6</v>
       </c>
@@ -19665,7 +19803,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J66" s="39" t="n"/>
+      <c r="J66" s="39" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K66" s="8" t="n">
         <v>18</v>
       </c>
@@ -19775,7 +19915,9 @@
           <t>HAR_NM_A_Belt_a</t>
         </is>
       </c>
-      <c r="D69" s="41" t="n"/>
+      <c r="D69" s="41" t="n">
+        <v>0.5</v>
+      </c>
       <c r="E69" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -19790,8 +19932,14 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="I69" s="44" t="n"/>
-      <c r="J69" s="39" t="n"/>
+      <c r="I69" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J69" s="39" t="n">
+        <v>0.5</v>
+      </c>
       <c r="K69" s="8" t="n">
         <v>16</v>
       </c>
@@ -19911,7 +20059,9 @@
           <t>HAR_LL_A_a</t>
         </is>
       </c>
-      <c r="D72" s="40" t="n"/>
+      <c r="D72" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E72" s="28" t="n">
         <v>1.3</v>
       </c>
@@ -19927,14 +20077,18 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J72" s="44" t="n"/>
+      <c r="J72" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K72" s="76" t="n">
         <v>20</v>
       </c>
       <c r="L72" s="76" t="n">
         <v>44</v>
       </c>
-      <c r="M72" s="8" t="n"/>
+      <c r="M72" s="8" t="n">
+        <v>1.3</v>
+      </c>
       <c r="N72" s="76" t="n">
         <v>80</v>
       </c>
@@ -19961,7 +20115,9 @@
           <t>HAR_LL_H_f</t>
         </is>
       </c>
-      <c r="D73" s="40" t="n"/>
+      <c r="D73" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E73" s="28" t="n">
         <v>1.3</v>
       </c>
@@ -19977,14 +20133,18 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J73" s="44" t="n"/>
+      <c r="J73" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K73" s="76" t="n">
         <v>18</v>
       </c>
       <c r="L73" s="76" t="n">
         <v>38</v>
       </c>
-      <c r="M73" s="8" t="n"/>
+      <c r="M73" s="8" t="n">
+        <v>1.3</v>
+      </c>
       <c r="N73" s="76" t="n">
         <v>40</v>
       </c>
@@ -20613,7 +20773,9 @@
           <t>HAR_IA_Armor_a</t>
         </is>
       </c>
-      <c r="D89" s="40" t="n"/>
+      <c r="D89" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E89" s="28" t="n">
         <v>1</v>
       </c>
@@ -20629,7 +20791,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J89" s="44" t="n"/>
+      <c r="J89" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K89" s="76" t="n">
         <v>16</v>
       </c>
@@ -20665,7 +20829,9 @@
           <t>HAR_IA_AH_a</t>
         </is>
       </c>
-      <c r="D90" s="40" t="n"/>
+      <c r="D90" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E90" s="28" t="n">
         <v>1</v>
       </c>
@@ -20681,7 +20847,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J90" s="44" t="n"/>
+      <c r="J90" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K90" s="76" t="n">
         <v>14</v>
       </c>
@@ -20715,7 +20883,9 @@
           <t>HAR_IA_AH_b</t>
         </is>
       </c>
-      <c r="D91" s="40" t="n"/>
+      <c r="D91" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E91" s="28" t="n">
         <v>2</v>
       </c>
@@ -20731,7 +20901,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J91" s="44" t="n"/>
+      <c r="J91" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K91" s="76" t="n">
         <v>28</v>
       </c>
@@ -20909,7 +21081,9 @@
           <t>HAR_IA_Armor_b</t>
         </is>
       </c>
-      <c r="D95" s="40" t="n"/>
+      <c r="D95" s="40" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E95" s="28" t="n">
         <v>2</v>
       </c>
@@ -20925,7 +21099,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J95" s="44" t="n"/>
+      <c r="J95" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K95" s="76" t="n">
         <v>24</v>
       </c>
@@ -21464,7 +21640,9 @@
       </c>
       <c r="E108" s="5" t="n"/>
       <c r="F108" s="5" t="n"/>
-      <c r="G108" s="41" t="n"/>
+      <c r="G108" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H108" s="33" t="n"/>
       <c r="I108" s="78" t="inlineStr">
         <is>
@@ -21476,7 +21654,9 @@
       </c>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
-      <c r="M108" s="8" t="n"/>
+      <c r="M108" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="N108" s="84" t="n">
         <v>1</v>
       </c>
@@ -21504,7 +21684,9 @@
       </c>
       <c r="E109" s="5" t="n"/>
       <c r="F109" s="5" t="n"/>
-      <c r="G109" s="41" t="n"/>
+      <c r="G109" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H109" s="33" t="n"/>
       <c r="I109" s="78" t="inlineStr">
         <is>
@@ -21516,7 +21698,9 @@
       </c>
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="n"/>
-      <c r="M109" s="8" t="n"/>
+      <c r="M109" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="N109" s="84" t="n">
         <v>1</v>
       </c>
@@ -21544,7 +21728,9 @@
       </c>
       <c r="E110" s="5" t="n"/>
       <c r="F110" s="5" t="n"/>
-      <c r="G110" s="41" t="n"/>
+      <c r="G110" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H110" s="33" t="n"/>
       <c r="I110" s="78" t="inlineStr">
         <is>
@@ -21556,7 +21742,9 @@
       </c>
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="n"/>
-      <c r="M110" s="8" t="n"/>
+      <c r="M110" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="N110" s="84" t="n">
         <v>1</v>
       </c>
@@ -21584,7 +21772,9 @@
       </c>
       <c r="E111" s="5" t="n"/>
       <c r="F111" s="5" t="n"/>
-      <c r="G111" s="41" t="n"/>
+      <c r="G111" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H111" s="33" t="n"/>
       <c r="I111" s="78" t="inlineStr">
         <is>
@@ -21596,7 +21786,9 @@
       </c>
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="n"/>
-      <c r="M111" s="8" t="n"/>
+      <c r="M111" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="N111" s="84" t="n">
         <v>10</v>
       </c>
@@ -21616,7 +21808,7 @@
       </c>
       <c r="C112" s="70" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_c</t>
+          <t>HAR_CO_Apparel_Head_c</t>
         </is>
       </c>
       <c r="D112" s="41" t="n">
@@ -21624,17 +21816,29 @@
       </c>
       <c r="E112" s="5" t="n"/>
       <c r="F112" s="5" t="n"/>
-      <c r="G112" s="41" t="n"/>
+      <c r="G112" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H112" s="33" t="n"/>
-      <c r="I112" s="44" t="n"/>
+      <c r="I112" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="J112" s="44" t="n">
         <v>0</v>
       </c>
       <c r="K112" s="8" t="n"/>
       <c r="L112" s="8" t="n"/>
-      <c r="M112" s="8" t="n"/>
-      <c r="N112" s="25" t="n"/>
-      <c r="O112" s="25" t="n"/>
+      <c r="M112" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N112" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O112" s="25" t="n">
+        <v>1</v>
+      </c>
       <c r="P112" s="52" t="n"/>
       <c r="Q112" s="52" t="n"/>
       <c r="R112" s="52" t="n"/>
@@ -21648,7 +21852,7 @@
       </c>
       <c r="C113" s="70" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_b</t>
+          <t>HAR_CO_Apparel_Head_b</t>
         </is>
       </c>
       <c r="D113" s="41" t="n">
@@ -21656,17 +21860,29 @@
       </c>
       <c r="E113" s="5" t="n"/>
       <c r="F113" s="5" t="n"/>
-      <c r="G113" s="41" t="n"/>
+      <c r="G113" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H113" s="33" t="n"/>
-      <c r="I113" s="44" t="n"/>
+      <c r="I113" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="J113" s="44" t="n">
         <v>0</v>
       </c>
       <c r="K113" s="8" t="n"/>
       <c r="L113" s="8" t="n"/>
-      <c r="M113" s="8" t="n"/>
-      <c r="N113" s="25" t="n"/>
-      <c r="O113" s="25" t="n"/>
+      <c r="M113" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N113" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O113" s="25" t="n">
+        <v>1</v>
+      </c>
       <c r="P113" s="52" t="n"/>
       <c r="Q113" s="52" t="n"/>
       <c r="R113" s="52" t="n"/>
@@ -21680,7 +21896,7 @@
       </c>
       <c r="C114" s="70" t="inlineStr">
         <is>
-          <t>HAR_CO_Apparel_head_a</t>
+          <t>HAR_CO_Apparel_Head_a</t>
         </is>
       </c>
       <c r="D114" s="41" t="n">
@@ -21688,17 +21904,29 @@
       </c>
       <c r="E114" s="5" t="n"/>
       <c r="F114" s="5" t="n"/>
-      <c r="G114" s="41" t="n"/>
+      <c r="G114" s="41" t="n">
+        <v>2</v>
+      </c>
       <c r="H114" s="33" t="n"/>
-      <c r="I114" s="44" t="n"/>
+      <c r="I114" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="J114" s="44" t="n">
         <v>0</v>
       </c>
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="8" t="n"/>
-      <c r="M114" s="8" t="n"/>
-      <c r="N114" s="25" t="n"/>
-      <c r="O114" s="25" t="n"/>
+      <c r="M114" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N114" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O114" s="25" t="n">
+        <v>1</v>
+      </c>
       <c r="P114" s="52" t="n"/>
       <c r="Q114" s="52" t="n"/>
       <c r="R114" s="52" t="n"/>
@@ -22669,7 +22897,9 @@
           <t>HAR_QL_A_a</t>
         </is>
       </c>
-      <c r="D137" s="41" t="n"/>
+      <c r="D137" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E137" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -22685,7 +22915,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J137" s="44" t="n"/>
+      <c r="J137" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K137" s="76" t="n">
         <v>24</v>
       </c>
@@ -22721,7 +22953,9 @@
           <t>HAR_QL_H_a</t>
         </is>
       </c>
-      <c r="D138" s="41" t="n"/>
+      <c r="D138" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E138" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -22737,7 +22971,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J138" s="44" t="n"/>
+      <c r="J138" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K138" s="76" t="n">
         <v>24</v>
       </c>
@@ -22768,10 +23004,12 @@
       </c>
       <c r="C139" s="70" t="inlineStr">
         <is>
-          <t>HAR_QA_S_a</t>
-        </is>
-      </c>
-      <c r="D139" s="41" t="n"/>
+          <t>HAR_QL_S_a</t>
+        </is>
+      </c>
+      <c r="D139" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E139" s="28" t="n">
         <v>0.5</v>
       </c>
@@ -22782,13 +23020,29 @@
         <v>0.5</v>
       </c>
       <c r="H139" s="33" t="n"/>
-      <c r="I139" s="44" t="n"/>
-      <c r="J139" s="44" t="n"/>
-      <c r="K139" s="8" t="n"/>
-      <c r="L139" s="8" t="n"/>
-      <c r="M139" s="8" t="n"/>
-      <c r="N139" s="25" t="n"/>
-      <c r="O139" s="25" t="n"/>
+      <c r="I139" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J139" s="44" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K139" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L139" s="8" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M139" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N139" s="25" t="n">
+        <v>40</v>
+      </c>
+      <c r="O139" s="25" t="n">
+        <v>10</v>
+      </c>
       <c r="P139" s="52" t="n"/>
       <c r="Q139" s="52" t="n"/>
       <c r="R139" s="52" t="n"/>
@@ -22847,7 +23101,9 @@
           <t>HAR_QL_T_a</t>
         </is>
       </c>
-      <c r="D141" s="41" t="n"/>
+      <c r="D141" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E141" s="28" t="n">
         <v>0.9</v>
       </c>
@@ -22863,14 +23119,18 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J141" s="44" t="n"/>
+      <c r="J141" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K141" s="84" t="n">
         <v>1</v>
       </c>
       <c r="L141" s="84" t="n">
         <v>1.5</v>
       </c>
-      <c r="M141" s="8" t="n"/>
+      <c r="M141" s="8" t="n">
+        <v>0.9</v>
+      </c>
       <c r="N141" s="84" t="n">
         <v>40</v>
       </c>
@@ -22893,7 +23153,9 @@
           <t>HAR_QL_S_b</t>
         </is>
       </c>
-      <c r="D142" s="41" t="n"/>
+      <c r="D142" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E142" s="28" t="n">
         <v>0.5</v>
       </c>
@@ -22909,14 +23171,18 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J142" s="44" t="n"/>
+      <c r="J142" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K142" s="84" t="n">
         <v>5</v>
       </c>
       <c r="L142" s="84" t="n">
         <v>7.5</v>
       </c>
-      <c r="M142" s="8" t="n"/>
+      <c r="M142" s="8" t="n">
+        <v>0.5</v>
+      </c>
       <c r="N142" s="84" t="n">
         <v>40</v>
       </c>
@@ -22939,7 +23205,9 @@
           <t>HAR_QL_O_b</t>
         </is>
       </c>
-      <c r="D143" s="41" t="n"/>
+      <c r="D143" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E143" s="28" t="n">
         <v>0.4</v>
       </c>
@@ -22964,7 +23232,9 @@
       <c r="L143" s="84" t="n">
         <v>12</v>
       </c>
-      <c r="M143" s="8" t="n"/>
+      <c r="M143" s="8" t="n">
+        <v>0.4</v>
+      </c>
       <c r="N143" s="84" t="n">
         <v>0.5</v>
       </c>
@@ -22987,7 +23257,9 @@
           <t>HAR_QL_O_a</t>
         </is>
       </c>
-      <c r="D144" s="41" t="n"/>
+      <c r="D144" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E144" s="28" t="n">
         <v>0.4</v>
       </c>
@@ -23012,7 +23284,9 @@
       <c r="L144" s="84" t="n">
         <v>12</v>
       </c>
-      <c r="M144" s="8" t="n"/>
+      <c r="M144" s="8" t="n">
+        <v>0.4</v>
+      </c>
       <c r="N144" s="84" t="n">
         <v>0.5</v>
       </c>
@@ -23035,7 +23309,9 @@
           <t>HAR_QL_O_c</t>
         </is>
       </c>
-      <c r="D145" s="41" t="n"/>
+      <c r="D145" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E145" s="28" t="n">
         <v>0.4</v>
       </c>
@@ -23060,7 +23336,9 @@
       <c r="L145" s="84" t="n">
         <v>12</v>
       </c>
-      <c r="M145" s="8" t="n"/>
+      <c r="M145" s="8" t="n">
+        <v>0.4</v>
+      </c>
       <c r="N145" s="84" t="n">
         <v>0.5</v>
       </c>
@@ -24702,7 +24980,9 @@
           <t>HAR_SA_Armor_a</t>
         </is>
       </c>
-      <c r="D185" s="41" t="n"/>
+      <c r="D185" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E185" s="28" t="n">
         <v>0.9</v>
       </c>
@@ -24717,8 +24997,14 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="I185" s="44" t="n"/>
-      <c r="J185" s="44" t="n"/>
+      <c r="I185" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J185" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K185" s="8" t="n">
         <v>16</v>
       </c>
@@ -24750,7 +25036,9 @@
           <t>HAR_SA_Heads_d</t>
         </is>
       </c>
-      <c r="D186" s="41" t="n"/>
+      <c r="D186" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E186" s="28" t="n">
         <v>0.9</v>
       </c>
@@ -24770,7 +25058,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J186" s="44" t="n"/>
+      <c r="J186" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K186" s="8" t="n">
         <v>18</v>
       </c>
@@ -24844,7 +25134,9 @@
           <t>HAR_SA_Shell_c</t>
         </is>
       </c>
-      <c r="D188" s="41" t="n"/>
+      <c r="D188" s="41" t="n">
+        <v>1</v>
+      </c>
       <c r="E188" s="28" t="n">
         <v>0.4</v>
       </c>
@@ -24859,8 +25151,14 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="I188" s="44" t="n"/>
-      <c r="J188" s="44" t="n"/>
+      <c r="I188" s="44" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J188" s="44" t="n">
+        <v>1</v>
+      </c>
       <c r="K188" s="8" t="n">
         <v>10</v>
       </c>
@@ -26338,7 +26636,9 @@
           <t>HAR_EL_Apparel_Armor_a</t>
         </is>
       </c>
-      <c r="D223" s="41" t="n"/>
+      <c r="D223" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E223" s="28" t="n">
         <v>1</v>
       </c>
@@ -26354,7 +26654,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J223" s="44" t="n"/>
+      <c r="J223" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K223" s="76" t="n">
         <v>18</v>
       </c>
@@ -26390,7 +26692,9 @@
           <t>HAR_EL_Apparel_Head_d</t>
         </is>
       </c>
-      <c r="D224" s="41" t="n"/>
+      <c r="D224" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E224" s="28" t="n">
         <v>1</v>
       </c>
@@ -26406,7 +26710,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J224" s="44" t="n"/>
+      <c r="J224" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K224" s="76" t="n">
         <v>16</v>
       </c>
@@ -27681,7 +27987,9 @@
           <t>HAR_ZC_Heads_d</t>
         </is>
       </c>
-      <c r="D258" s="41" t="n"/>
+      <c r="D258" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E258" s="28" t="n">
         <v>1</v>
       </c>
@@ -27697,7 +28005,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J258" s="44" t="n"/>
+      <c r="J258" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K258" s="76" t="n">
         <v>18</v>
       </c>
@@ -27731,7 +28041,9 @@
           <t>HAR_ZC_Heads_e</t>
         </is>
       </c>
-      <c r="D259" s="41" t="n"/>
+      <c r="D259" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E259" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -27747,7 +28059,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J259" s="44" t="n"/>
+      <c r="J259" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K259" s="76" t="n">
         <v>24</v>
       </c>
@@ -27941,7 +28255,9 @@
           <t>HAR_ZC_Shell_e</t>
         </is>
       </c>
-      <c r="D264" s="41" t="n"/>
+      <c r="D264" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E264" s="28" t="n">
         <v>1</v>
       </c>
@@ -27957,7 +28273,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J264" s="44" t="n"/>
+      <c r="J264" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K264" s="76" t="n">
         <v>18</v>
       </c>
@@ -27989,7 +28307,9 @@
           <t>HAR_ZC_Shell_f</t>
         </is>
       </c>
-      <c r="D265" s="41" t="n"/>
+      <c r="D265" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E265" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -28005,7 +28325,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J265" s="44" t="n"/>
+      <c r="J265" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K265" s="76" t="n">
         <v>24</v>
       </c>
@@ -28157,7 +28479,9 @@
           <t>HAR_ZC_Tops_d</t>
         </is>
       </c>
-      <c r="D269" s="41" t="n"/>
+      <c r="D269" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E269" s="28" t="n">
         <v>1</v>
       </c>
@@ -28173,7 +28497,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J269" s="44" t="n"/>
+      <c r="J269" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K269" s="76" t="n">
         <v>18</v>
       </c>
@@ -28209,7 +28535,9 @@
           <t>HAR_ZC_Tops_e</t>
         </is>
       </c>
-      <c r="D270" s="41" t="n"/>
+      <c r="D270" s="41" t="n">
+        <v>0.1</v>
+      </c>
       <c r="E270" s="28" t="n">
         <v>1.5</v>
       </c>
@@ -28225,7 +28553,9 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="J270" s="44" t="n"/>
+      <c r="J270" s="44" t="n">
+        <v>0.1</v>
+      </c>
       <c r="K270" s="76" t="n">
         <v>24</v>
       </c>

</xml_diff>

<commit_message>
Add Outerm CE patches
</commit_message>
<xml_diff>
--- a/RimWorld CE Ayameduki Race Patching and Stats - reviewed.xlsx
+++ b/RimWorld CE Ayameduki Race Patching and Stats - reviewed.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="38280" yWindow="15" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Armor Stats (Clean)" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +12,7 @@
     <sheet name="Discrepancies" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,41 +30,49 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00111827"/>
+      <name val="Calibri"/>
+      <color rgb="FF111827"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00111827"/>
+      <color rgb="FF111827"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <color rgb="00111827"/>
+      <color rgb="FF111827"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="16">
@@ -77,72 +84,72 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00334155"/>
+        <fgColor rgb="FF334155"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F59E0B"/>
+        <fgColor rgb="FFF59E0B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
+        <fgColor rgb="FF2563EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006D4C41"/>
+        <fgColor rgb="FF6D4C41"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003E2723"/>
+        <fgColor rgb="FF3E2723"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFEBE9"/>
+        <fgColor rgb="FFEFEBE9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3BF"/>
+        <fgColor rgb="FFFFF3BF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
+        <fgColor rgb="FFFFCDD2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE0B2"/>
+        <fgColor rgb="FFFFE0B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,36 +163,44 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </left>
       <right style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </right>
       <top style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="FFE2E8F0"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0BEC5"/>
+        <color rgb="FFB0BEC5"/>
       </left>
       <right style="thin">
-        <color rgb="00B0BEC5"/>
+        <color rgb="FFB0BEC5"/>
       </right>
       <top style="thin">
-        <color rgb="00B0BEC5"/>
+        <color rgb="FFB0BEC5"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0BEC5"/>
+        <color rgb="FFB0BEC5"/>
       </bottom>
+      <diagonal/>
     </border>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3"/>
   </cellStyleXfs>
   <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -281,7 +296,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -710,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V264"/>
+  <dimension ref="A1:V266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -722,14 +737,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="10" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
@@ -737,7 +745,7 @@
     <col width="10" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Mod Name</t>
@@ -16472,7 +16480,9 @@
       <c r="J246" s="11" t="n"/>
       <c r="K246" s="11" t="n"/>
       <c r="L246" s="11" t="n"/>
-      <c r="M246" s="12" t="n"/>
+      <c r="M246" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N246" s="13" t="n"/>
       <c r="O246" s="13" t="n"/>
       <c r="P246" s="13" t="n"/>
@@ -16522,7 +16532,9 @@
       <c r="J247" s="11" t="n"/>
       <c r="K247" s="11" t="n"/>
       <c r="L247" s="11" t="n"/>
-      <c r="M247" s="12" t="n"/>
+      <c r="M247" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N247" s="13" t="n"/>
       <c r="O247" s="13" t="n"/>
       <c r="P247" s="13" t="n"/>
@@ -16572,7 +16584,9 @@
       <c r="J248" s="11" t="n"/>
       <c r="K248" s="11" t="n"/>
       <c r="L248" s="11" t="n"/>
-      <c r="M248" s="12" t="n"/>
+      <c r="M248" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N248" s="13" t="n"/>
       <c r="O248" s="13" t="n"/>
       <c r="P248" s="13" t="n"/>
@@ -16622,7 +16636,9 @@
       <c r="J249" s="11" t="n"/>
       <c r="K249" s="11" t="n"/>
       <c r="L249" s="11" t="n"/>
-      <c r="M249" s="12" t="n"/>
+      <c r="M249" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="N249" s="13" t="n"/>
       <c r="O249" s="13" t="n"/>
       <c r="P249" s="13" t="n"/>
@@ -16672,7 +16688,9 @@
       <c r="J250" s="11" t="n"/>
       <c r="K250" s="11" t="n"/>
       <c r="L250" s="11" t="n"/>
-      <c r="M250" s="12" t="n"/>
+      <c r="M250" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="N250" s="13" t="n"/>
       <c r="O250" s="13" t="n"/>
       <c r="P250" s="13" t="n"/>
@@ -16722,7 +16740,9 @@
       <c r="J251" s="11" t="n"/>
       <c r="K251" s="11" t="n"/>
       <c r="L251" s="11" t="n"/>
-      <c r="M251" s="12" t="n"/>
+      <c r="M251" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="N251" s="13" t="n"/>
       <c r="O251" s="13" t="n"/>
       <c r="P251" s="13" t="n"/>
@@ -16772,7 +16792,9 @@
       <c r="J252" s="11" t="n"/>
       <c r="K252" s="11" t="n"/>
       <c r="L252" s="11" t="n"/>
-      <c r="M252" s="12" t="n"/>
+      <c r="M252" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="N252" s="13" t="n"/>
       <c r="O252" s="13" t="n"/>
       <c r="P252" s="13" t="n"/>
@@ -16822,7 +16844,9 @@
       <c r="J253" s="11" t="n"/>
       <c r="K253" s="11" t="n"/>
       <c r="L253" s="11" t="n"/>
-      <c r="M253" s="12" t="n"/>
+      <c r="M253" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="N253" s="13" t="n"/>
       <c r="O253" s="13" t="n"/>
       <c r="P253" s="13" t="n"/>
@@ -16872,7 +16896,9 @@
       <c r="J254" s="11" t="n"/>
       <c r="K254" s="11" t="n"/>
       <c r="L254" s="11" t="n"/>
-      <c r="M254" s="12" t="n"/>
+      <c r="M254" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="N254" s="13" t="n"/>
       <c r="O254" s="13" t="n"/>
       <c r="P254" s="13" t="n"/>
@@ -16922,7 +16948,9 @@
       <c r="J255" s="11" t="n"/>
       <c r="K255" s="11" t="n"/>
       <c r="L255" s="11" t="n"/>
-      <c r="M255" s="12" t="n"/>
+      <c r="M255" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="N255" s="13" t="n"/>
       <c r="O255" s="13" t="n"/>
       <c r="P255" s="13" t="n"/>
@@ -16972,7 +17000,9 @@
       <c r="J256" s="11" t="n"/>
       <c r="K256" s="11" t="n"/>
       <c r="L256" s="11" t="n"/>
-      <c r="M256" s="12" t="n"/>
+      <c r="M256" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="N256" s="13" t="n"/>
       <c r="O256" s="13" t="n"/>
       <c r="P256" s="13" t="n"/>
@@ -17022,7 +17052,9 @@
       <c r="J257" s="11" t="n"/>
       <c r="K257" s="11" t="n"/>
       <c r="L257" s="11" t="n"/>
-      <c r="M257" s="12" t="n"/>
+      <c r="M257" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="N257" s="13" t="n"/>
       <c r="O257" s="13" t="n"/>
       <c r="P257" s="13" t="n"/>
@@ -17072,7 +17104,9 @@
       <c r="J258" s="11" t="n"/>
       <c r="K258" s="11" t="n"/>
       <c r="L258" s="11" t="n"/>
-      <c r="M258" s="12" t="n"/>
+      <c r="M258" s="12" t="n">
+        <v>5</v>
+      </c>
       <c r="N258" s="13" t="n"/>
       <c r="O258" s="13" t="n"/>
       <c r="P258" s="13" t="n"/>
@@ -17122,7 +17156,9 @@
       <c r="J259" s="11" t="n"/>
       <c r="K259" s="11" t="n"/>
       <c r="L259" s="11" t="n"/>
-      <c r="M259" s="12" t="n"/>
+      <c r="M259" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N259" s="13" t="n"/>
       <c r="O259" s="13" t="n"/>
       <c r="P259" s="13" t="n"/>
@@ -17172,7 +17208,9 @@
       <c r="J260" s="11" t="n"/>
       <c r="K260" s="11" t="n"/>
       <c r="L260" s="11" t="n"/>
-      <c r="M260" s="12" t="n"/>
+      <c r="M260" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N260" s="13" t="n"/>
       <c r="O260" s="13" t="n"/>
       <c r="P260" s="13" t="n"/>
@@ -17222,7 +17260,9 @@
       <c r="J261" s="11" t="n"/>
       <c r="K261" s="11" t="n"/>
       <c r="L261" s="11" t="n"/>
-      <c r="M261" s="12" t="n"/>
+      <c r="M261" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N261" s="13" t="n"/>
       <c r="O261" s="13" t="n"/>
       <c r="P261" s="13" t="n"/>
@@ -17272,7 +17312,9 @@
       <c r="J262" s="11" t="n"/>
       <c r="K262" s="11" t="n"/>
       <c r="L262" s="11" t="n"/>
-      <c r="M262" s="12" t="n"/>
+      <c r="M262" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N262" s="13" t="n"/>
       <c r="O262" s="13" t="n"/>
       <c r="P262" s="13" t="n"/>
@@ -17322,7 +17364,9 @@
       <c r="J263" s="11" t="n"/>
       <c r="K263" s="11" t="n"/>
       <c r="L263" s="11" t="n"/>
-      <c r="M263" s="12" t="n"/>
+      <c r="M263" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N263" s="13" t="n"/>
       <c r="O263" s="13" t="n"/>
       <c r="P263" s="13" t="n"/>
@@ -17372,7 +17416,9 @@
       <c r="J264" s="11" t="n"/>
       <c r="K264" s="11" t="n"/>
       <c r="L264" s="11" t="n"/>
-      <c r="M264" s="12" t="n"/>
+      <c r="M264" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="N264" s="13" t="n"/>
       <c r="O264" s="13" t="n"/>
       <c r="P264" s="13" t="n"/>
@@ -17382,6 +17428,164 @@
       <c r="T264" s="13" t="n"/>
       <c r="U264" s="13" t="n"/>
       <c r="V264" s="14" t="n"/>
+    </row>
+    <row r="265" ht="12" customHeight="1">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>Outerm</t>
+        </is>
+      </c>
+      <c r="B265" s="5" t="inlineStr">
+        <is>
+          <t>??????????</t>
+        </is>
+      </c>
+      <c r="C265" s="6" t="inlineStr">
+        <is>
+          <t>HAR_OT_Apparel_T_Armor_a</t>
+        </is>
+      </c>
+      <c r="D265" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E265" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F265" s="4" t="inlineStr">
+        <is>
+          <t>CE Bulk, CE Worn Bulk, CE Carry Weight, CE Bulk Capacity, CE Sharp, CE Blunt, CE Heat, CE Material</t>
+        </is>
+      </c>
+      <c r="G265" s="9" t="inlineStr">
+        <is>
+          <t>Added from source defs; CE values derived from exact-stat power armor analogs</t>
+        </is>
+      </c>
+      <c r="H265" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Outerm_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I265" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J265" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K265" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L265" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M265" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N265" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="O265" s="13" t="n">
+        <v>42</v>
+      </c>
+      <c r="P265" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q265" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="R265" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="S265" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="T265" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="U265" s="13" t="n"/>
+      <c r="V265" s="14" t="n"/>
+    </row>
+    <row r="266" ht="12" customHeight="1">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>Outerm</t>
+        </is>
+      </c>
+      <c r="B266" s="5" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+      <c r="C266" s="6" t="inlineStr">
+        <is>
+          <t>HAR_OT_Apparel_H_z</t>
+        </is>
+      </c>
+      <c r="D266" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E266" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F266" s="4" t="inlineStr">
+        <is>
+          <t>CE Bulk, CE Worn Bulk, CE Night Vision, CE Sharp, CE Blunt, CE Heat, CE Material</t>
+        </is>
+      </c>
+      <c r="G266" s="9" t="inlineStr">
+        <is>
+          <t>Added from source defs; CE values derived from exact-stat power armor analogs</t>
+        </is>
+      </c>
+      <c r="H266" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Outerm_Apparel.xml</t>
+        </is>
+      </c>
+      <c r="I266" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J266" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K266" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L266" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M266" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N266" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="O266" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="P266" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q266" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="R266" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="S266" s="13" t="n"/>
+      <c r="T266" s="13" t="n"/>
+      <c r="U266" s="13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="V266" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17403,50 +17607,19 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="10" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="11" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
-    <col width="11" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="11" customWidth="1" min="30" max="30"/>
-    <col width="11" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="11" customWidth="1" min="33" max="33"/>
-    <col width="11" customWidth="1" min="34" max="34"/>
-    <col width="11" customWidth="1" min="35" max="35"/>
-    <col width="11" customWidth="1" min="36" max="36"/>
-    <col width="11" customWidth="1" min="37" max="37"/>
-    <col width="11" customWidth="1" min="38" max="38"/>
-    <col width="11" customWidth="1" min="39" max="39"/>
-    <col width="11" customWidth="1" min="40" max="40"/>
-    <col width="18" customWidth="1" min="41" max="41"/>
-    <col width="18" customWidth="1" min="42" max="42"/>
-    <col width="18" customWidth="1" min="43" max="43"/>
+    <col width="11" customWidth="1" min="21" max="40"/>
+    <col width="18" customWidth="1" min="41" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="32.1" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Mod Name</t>
@@ -21274,16 +21447,24 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>CE Extra Effects, CE Melee AP Blunt, CE Melee AP Sharp, CE Melee Cooldown, CE Melee Power</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>No current CE patch for this item</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="n"/>
+          <t>Derived from source mod stats and CE melee baselines</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Weapons.xml</t>
+        </is>
+      </c>
       <c r="J33" s="10" t="n">
         <v>15</v>
       </c>
@@ -21303,10 +21484,18 @@
       <c r="T33" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="U33" s="12" t="n"/>
-      <c r="V33" s="12" t="n"/>
-      <c r="W33" s="12" t="n"/>
-      <c r="X33" s="12" t="n"/>
+      <c r="U33" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="V33" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="W33" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="X33" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="Y33" s="12" t="n"/>
       <c r="Z33" s="12" t="n"/>
       <c r="AA33" s="12" t="n"/>
@@ -21325,7 +21514,11 @@
       <c r="AN33" s="12" t="n"/>
       <c r="AO33" s="18" t="n"/>
       <c r="AP33" s="18" t="n"/>
-      <c r="AQ33" s="18" t="n"/>
+      <c r="AQ33" s="18" t="inlineStr">
+        <is>
+          <t>Growing weapon; MoveSpeed +2, MeleeHitChance +3, MeleeDodgeChance +3</t>
+        </is>
+      </c>
       <c r="AR33" s="14" t="n"/>
     </row>
     <row r="34" ht="12" customHeight="1">
@@ -21356,16 +21549,24 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>CE Extra Effects, CE Melee AP Blunt, CE Melee AP Sharp, CE Melee Cooldown, CE Melee Power</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>No current CE patch for this item</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="n"/>
+          <t>Derived from source mod stats and CE melee baselines</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Weapons.xml</t>
+        </is>
+      </c>
       <c r="J34" s="10" t="n">
         <v>15</v>
       </c>
@@ -21385,10 +21586,18 @@
       <c r="T34" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="U34" s="12" t="n"/>
-      <c r="V34" s="12" t="n"/>
-      <c r="W34" s="12" t="n"/>
-      <c r="X34" s="12" t="n"/>
+      <c r="U34" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="V34" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="W34" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="X34" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="Y34" s="12" t="n"/>
       <c r="Z34" s="12" t="n"/>
       <c r="AA34" s="12" t="n"/>
@@ -21407,7 +21616,11 @@
       <c r="AN34" s="12" t="n"/>
       <c r="AO34" s="18" t="n"/>
       <c r="AP34" s="18" t="n"/>
-      <c r="AQ34" s="18" t="n"/>
+      <c r="AQ34" s="18" t="inlineStr">
+        <is>
+          <t>Growing weapon; ArmorRating_Blunt +1, MeleeHitChance +3, MeleeDodgeChance +3</t>
+        </is>
+      </c>
       <c r="AR34" s="14" t="n"/>
     </row>
     <row r="35" ht="12" customHeight="1">
@@ -21438,16 +21651,24 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>CE Extra Effects, CE Melee AP Blunt, CE Melee AP Sharp, CE Melee Cooldown, CE Melee Power</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>No current CE patch for this item</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="n"/>
+          <t>Derived from source mod stats and CE melee baselines</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Weapons.xml</t>
+        </is>
+      </c>
       <c r="J35" s="10" t="n">
         <v>15</v>
       </c>
@@ -21467,10 +21688,18 @@
       <c r="T35" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="U35" s="12" t="n"/>
-      <c r="V35" s="12" t="n"/>
-      <c r="W35" s="12" t="n"/>
-      <c r="X35" s="12" t="n"/>
+      <c r="U35" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="V35" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="W35" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="X35" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="Y35" s="12" t="n"/>
       <c r="Z35" s="12" t="n"/>
       <c r="AA35" s="12" t="n"/>
@@ -21489,7 +21718,11 @@
       <c r="AN35" s="12" t="n"/>
       <c r="AO35" s="18" t="n"/>
       <c r="AP35" s="18" t="n"/>
-      <c r="AQ35" s="18" t="n"/>
+      <c r="AQ35" s="18" t="inlineStr">
+        <is>
+          <t>Growing weapon; ArmorRating_Sharp +1, MeleeHitChance +3, MeleeDodgeChance +3</t>
+        </is>
+      </c>
       <c r="AR35" s="14" t="n"/>
     </row>
     <row r="36" ht="12" customHeight="1">
@@ -21520,16 +21753,24 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>CE Ammo Set, CE Bulk, CE Burst, CE Extra Effects, CE Magazine, CE Mass, CE Melee AP Blunt, CE Melee AP Sharp, CE Melee Cooldown, CE Melee Power, CE Projectile, CE Range, CE Ranged AP Blunt, CE Ranged AP Sharp, CE Ranged Cooldown, CE Ranged Damage, CE Recoil, CE Reload, CE Shot Spread, CE Sights, CE Sway, CE Ticks/Burst, CE Warmup</t>
+        </is>
+      </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>No current CE patch for this item</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="n"/>
+          <t>Derived from source mod stats and CE 5.56 caliber baselines</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Weapons.xml; Patches/Outerm/Ammo/Projectiles.xml</t>
+        </is>
+      </c>
       <c r="J36" s="10" t="n">
         <v>9</v>
       </c>
@@ -21561,29 +21802,81 @@
       <c r="T36" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="U36" s="12" t="n"/>
-      <c r="V36" s="12" t="n"/>
-      <c r="W36" s="12" t="n"/>
-      <c r="X36" s="12" t="n"/>
-      <c r="Y36" s="12" t="n"/>
-      <c r="Z36" s="12" t="n"/>
-      <c r="AA36" s="12" t="n"/>
-      <c r="AB36" s="12" t="n"/>
-      <c r="AC36" s="12" t="n"/>
-      <c r="AD36" s="12" t="n"/>
-      <c r="AE36" s="12" t="n"/>
-      <c r="AF36" s="12" t="n"/>
-      <c r="AG36" s="12" t="n"/>
-      <c r="AH36" s="12" t="n"/>
-      <c r="AI36" s="12" t="n"/>
-      <c r="AJ36" s="12" t="n"/>
-      <c r="AK36" s="12" t="n"/>
-      <c r="AL36" s="12" t="n"/>
-      <c r="AM36" s="12" t="n"/>
-      <c r="AN36" s="12" t="n"/>
-      <c r="AO36" s="18" t="n"/>
-      <c r="AP36" s="18" t="n"/>
-      <c r="AQ36" s="18" t="n"/>
+      <c r="U36" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="V36" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="X36" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y36" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z36" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA36" s="12" t="n">
+        <v>34.18</v>
+      </c>
+      <c r="AB36" s="12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AC36" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="AD36" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AE36" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF36" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG36" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="AH36" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AI36" s="12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AJ36" s="12" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AK36" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL36" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AM36" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="AN36" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AO36" s="18" t="inlineStr">
+        <is>
+          <t>AmmoSet_HAR_OT_556x45mmNATO_Toxic</t>
+        </is>
+      </c>
+      <c r="AP36" s="18" t="inlineStr">
+        <is>
+          <t>HAR_OT_Bullet_556x45mmNATO_FMJ_Toxic</t>
+        </is>
+      </c>
+      <c r="AQ36" s="18" t="inlineStr">
+        <is>
+          <t>Uses standard 5.56x45 NATO ammo defs with toxic projectile mapping</t>
+        </is>
+      </c>
       <c r="AR36" s="14" t="n"/>
     </row>
     <row r="37" ht="12" customHeight="1">
@@ -21614,16 +21907,24 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="n"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>CE Ammo Set, CE Bulk, CE Burst, CE Extra Effects, CE Magazine, CE Mass, CE Melee AP Blunt, CE Melee AP Sharp, CE Melee Cooldown, CE Melee Power, CE Projectile, CE Range, CE Ranged AP Blunt, CE Ranged AP Sharp, CE Ranged Cooldown, CE Ranged Damage, CE Recoil, CE Reload, CE Shot Spread, CE Sights, CE Sway, CE Ticks/Burst, CE Warmup</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>No current CE patch for this item</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="n"/>
+          <t>Derived from source mod stats and CE 7.62 caliber baselines</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Patches/Outerm/ThingDefs_Misc/Weapons.xml; Patches/Outerm/Ammo/Projectiles.xml</t>
+        </is>
+      </c>
       <c r="J37" s="10" t="n">
         <v>9</v>
       </c>
@@ -21655,29 +21956,81 @@
       <c r="T37" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="U37" s="12" t="n"/>
-      <c r="V37" s="12" t="n"/>
-      <c r="W37" s="12" t="n"/>
-      <c r="X37" s="12" t="n"/>
-      <c r="Y37" s="12" t="n"/>
-      <c r="Z37" s="12" t="n"/>
-      <c r="AA37" s="12" t="n"/>
-      <c r="AB37" s="12" t="n"/>
-      <c r="AC37" s="12" t="n"/>
-      <c r="AD37" s="12" t="n"/>
-      <c r="AE37" s="12" t="n"/>
-      <c r="AF37" s="12" t="n"/>
-      <c r="AG37" s="12" t="n"/>
-      <c r="AH37" s="12" t="n"/>
-      <c r="AI37" s="12" t="n"/>
-      <c r="AJ37" s="12" t="n"/>
-      <c r="AK37" s="12" t="n"/>
-      <c r="AL37" s="12" t="n"/>
-      <c r="AM37" s="12" t="n"/>
-      <c r="AN37" s="12" t="n"/>
-      <c r="AO37" s="18" t="n"/>
-      <c r="AP37" s="18" t="n"/>
-      <c r="AQ37" s="18" t="n"/>
+      <c r="U37" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="V37" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="X37" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y37" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z37" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="AA37" s="12" t="n">
+        <v>66.72</v>
+      </c>
+      <c r="AB37" s="12" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AC37" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="AD37" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="AE37" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF37" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG37" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH37" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AI37" s="12" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AJ37" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AK37" s="12" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AL37" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM37" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN37" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO37" s="18" t="inlineStr">
+        <is>
+          <t>AmmoSet_HAR_OT_762x51mmNATO_Toxic</t>
+        </is>
+      </c>
+      <c r="AP37" s="18" t="inlineStr">
+        <is>
+          <t>HAR_OT_Bullet_762x51mmNATO_FMJ_Toxic</t>
+        </is>
+      </c>
+      <c r="AQ37" s="18" t="inlineStr">
+        <is>
+          <t>Uses standard 7.62x51 NATO ammo defs with toxic projectile mapping; no snapshot</t>
+        </is>
+      </c>
       <c r="AR37" s="14" t="n"/>
     </row>
   </sheetData>
@@ -21695,12 +22048,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="2" max="4"/>
+    <col width="12" customWidth="1" min="5" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21904,7 +22253,7 @@
     <col width="48" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="56.25" customHeight="1">
       <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Workbook Review Summary</t>
@@ -22048,7 +22397,7 @@
       <c r="I8" s="23" t="n"/>
       <c r="J8" s="23" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Category</t>
@@ -22100,7 +22449,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="25.5" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22146,7 +22495,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="25.5" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22192,7 +22541,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22238,7 +22587,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22284,7 +22633,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="25.5" customHeight="1">
       <c r="A14" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22330,7 +22679,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="25.5" customHeight="1">
       <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22376,7 +22725,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="25.5" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22422,7 +22771,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22468,7 +22817,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="25.5" customHeight="1">
       <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22514,7 +22863,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="25.5" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22560,7 +22909,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="25.5" customHeight="1">
       <c r="A20" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22606,7 +22955,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="25.5" customHeight="1">
       <c r="A21" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22652,7 +23001,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="25.5" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22698,7 +23047,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="25.5" customHeight="1">
       <c r="A23" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22744,7 +23093,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="25.5" customHeight="1">
       <c r="A24" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22790,7 +23139,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="25.5" customHeight="1">
       <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22836,7 +23185,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="25.5" customHeight="1">
       <c r="A26" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22882,7 +23231,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="25.5" customHeight="1">
       <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -22928,7 +23277,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="25.5" customHeight="1">
       <c r="A28" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -22974,7 +23323,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="25.5" customHeight="1">
       <c r="A29" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23020,7 +23369,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="25.5" customHeight="1">
       <c r="A30" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23066,7 +23415,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="25.5" customHeight="1">
       <c r="A31" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23112,7 +23461,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="25.5" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -23158,7 +23507,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="25.5" customHeight="1">
       <c r="A33" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23204,7 +23553,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="25.5" customHeight="1">
       <c r="A34" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23250,7 +23599,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="25.5" customHeight="1">
       <c r="A35" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23296,7 +23645,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="25.5" customHeight="1">
       <c r="A36" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23342,7 +23691,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="25.5" customHeight="1">
       <c r="A37" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -23388,7 +23737,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="25.5" customHeight="1">
       <c r="A38" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23434,7 +23783,7 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="25.5" customHeight="1">
       <c r="A39" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23480,7 +23829,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="25.5" customHeight="1">
       <c r="A40" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23526,7 +23875,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="25.5" customHeight="1">
       <c r="A41" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23572,7 +23921,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="25.5" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -23618,7 +23967,7 @@
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="25.5" customHeight="1">
       <c r="A43" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23664,7 +24013,7 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="25.5" customHeight="1">
       <c r="A44" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23710,7 +24059,7 @@
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="25.5" customHeight="1">
       <c r="A45" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23756,7 +24105,7 @@
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="25.5" customHeight="1">
       <c r="A46" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23802,7 +24151,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="25.5" customHeight="1">
       <c r="A47" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23848,7 +24197,7 @@
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="25.5" customHeight="1">
       <c r="A48" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -23894,7 +24243,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="25.5" customHeight="1">
       <c r="A49" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23940,7 +24289,7 @@
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="25.5" customHeight="1">
       <c r="A50" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -23986,7 +24335,7 @@
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="25.5" customHeight="1">
       <c r="A51" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24032,7 +24381,7 @@
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="25.5" customHeight="1">
       <c r="A52" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24078,7 +24427,7 @@
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="25.5" customHeight="1">
       <c r="A53" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24124,7 +24473,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="25.5" customHeight="1">
       <c r="A54" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -24170,7 +24519,7 @@
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="25.5" customHeight="1">
       <c r="A55" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24216,7 +24565,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="25.5" customHeight="1">
       <c r="A56" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24262,7 +24611,7 @@
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="25.5" customHeight="1">
       <c r="A57" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24308,7 +24657,7 @@
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="25.5" customHeight="1">
       <c r="A58" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24354,7 +24703,7 @@
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="25.5" customHeight="1">
       <c r="A59" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24400,7 +24749,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="25.5" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -24446,7 +24795,7 @@
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="25.5" customHeight="1">
       <c r="A61" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24492,7 +24841,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="25.5" customHeight="1">
       <c r="A62" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24538,7 +24887,7 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="25.5" customHeight="1">
       <c r="A63" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24584,7 +24933,7 @@
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="25.5" customHeight="1">
       <c r="A64" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24630,7 +24979,7 @@
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="25.5" customHeight="1">
       <c r="A65" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -24676,7 +25025,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="25.5" customHeight="1">
       <c r="A66" s="29" t="inlineStr">
         <is>
           <t>Patch flag cleared</t>
@@ -24718,7 +25067,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="25.5" customHeight="1">
       <c r="A67" s="29" t="inlineStr">
         <is>
           <t>Patch flag cleared</t>
@@ -24760,7 +25109,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="25.5" customHeight="1">
       <c r="A68" s="29" t="inlineStr">
         <is>
           <t>Patch flag cleared</t>
@@ -24802,7 +25151,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="25.5" customHeight="1">
       <c r="A69" s="29" t="inlineStr">
         <is>
           <t>Patch flag cleared</t>
@@ -24844,7 +25193,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="25.5" customHeight="1">
       <c r="A70" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24894,7 +25243,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="25.5" customHeight="1">
       <c r="A71" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24944,7 +25293,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="25.5" customHeight="1">
       <c r="A72" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -24994,7 +25343,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="25.5" customHeight="1">
       <c r="A73" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -25044,7 +25393,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="25.5" customHeight="1">
       <c r="A74" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25090,7 +25439,7 @@
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="25.5" customHeight="1">
       <c r="A75" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25136,7 +25485,7 @@
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="25.5" customHeight="1">
       <c r="A76" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25182,7 +25531,7 @@
         </is>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="25.5" customHeight="1">
       <c r="A77" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25228,7 +25577,7 @@
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="25.5" customHeight="1">
       <c r="A78" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25274,7 +25623,7 @@
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="25.5" customHeight="1">
       <c r="A79" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25320,7 +25669,7 @@
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="25.5" customHeight="1">
       <c r="A80" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25366,7 +25715,7 @@
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="25.5" customHeight="1">
       <c r="A81" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -25416,7 +25765,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="25.5" customHeight="1">
       <c r="A82" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25462,7 +25811,7 @@
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="25.5" customHeight="1">
       <c r="A83" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25508,7 +25857,7 @@
         </is>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="25.5" customHeight="1">
       <c r="A84" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25554,7 +25903,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="25.5" customHeight="1">
       <c r="A85" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25600,7 +25949,7 @@
         </is>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="25.5" customHeight="1">
       <c r="A86" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25646,7 +25995,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="25.5" customHeight="1">
       <c r="A87" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25692,7 +26041,7 @@
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="25.5" customHeight="1">
       <c r="A88" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25738,7 +26087,7 @@
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="25.5" customHeight="1">
       <c r="A89" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25784,7 +26133,7 @@
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="25.5" customHeight="1">
       <c r="A90" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25830,7 +26179,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="25.5" customHeight="1">
       <c r="A91" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25876,7 +26225,7 @@
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="25.5" customHeight="1">
       <c r="A92" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25922,7 +26271,7 @@
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="25.5" customHeight="1">
       <c r="A93" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -25968,7 +26317,7 @@
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="25.5" customHeight="1">
       <c r="A94" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26014,7 +26363,7 @@
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="25.5" customHeight="1">
       <c r="A95" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26060,7 +26409,7 @@
         </is>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="25.5" customHeight="1">
       <c r="A96" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26106,7 +26455,7 @@
         </is>
       </c>
     </row>
-    <row r="97">
+    <row r="97" ht="25.5" customHeight="1">
       <c r="A97" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26152,7 +26501,7 @@
         </is>
       </c>
     </row>
-    <row r="98">
+    <row r="98" ht="25.5" customHeight="1">
       <c r="A98" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26198,7 +26547,7 @@
         </is>
       </c>
     </row>
-    <row r="99">
+    <row r="99" ht="25.5" customHeight="1">
       <c r="A99" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26244,7 +26593,7 @@
         </is>
       </c>
     </row>
-    <row r="100">
+    <row r="100" ht="25.5" customHeight="1">
       <c r="A100" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26290,7 +26639,7 @@
         </is>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="25.5" customHeight="1">
       <c r="A101" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26336,7 +26685,7 @@
         </is>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="25.5" customHeight="1">
       <c r="A102" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26382,7 +26731,7 @@
         </is>
       </c>
     </row>
-    <row r="103">
+    <row r="103" ht="25.5" customHeight="1">
       <c r="A103" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26428,7 +26777,7 @@
         </is>
       </c>
     </row>
-    <row r="104">
+    <row r="104" ht="25.5" customHeight="1">
       <c r="A104" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26474,7 +26823,7 @@
         </is>
       </c>
     </row>
-    <row r="105">
+    <row r="105" ht="25.5" customHeight="1">
       <c r="A105" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26520,7 +26869,7 @@
         </is>
       </c>
     </row>
-    <row r="106">
+    <row r="106" ht="25.5" customHeight="1">
       <c r="A106" s="27" t="inlineStr">
         <is>
           <t>Value corrected</t>
@@ -26566,7 +26915,7 @@
         </is>
       </c>
     </row>
-    <row r="107">
+    <row r="107" ht="25.5" customHeight="1">
       <c r="A107" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26612,7 +26961,7 @@
         </is>
       </c>
     </row>
-    <row r="108">
+    <row r="108" ht="25.5" customHeight="1">
       <c r="A108" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26658,7 +27007,7 @@
         </is>
       </c>
     </row>
-    <row r="109">
+    <row r="109" ht="25.5" customHeight="1">
       <c r="A109" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26704,7 +27053,7 @@
         </is>
       </c>
     </row>
-    <row r="110">
+    <row r="110" ht="25.5" customHeight="1">
       <c r="A110" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26750,7 +27099,7 @@
         </is>
       </c>
     </row>
-    <row r="111">
+    <row r="111" ht="25.5" customHeight="1">
       <c r="A111" s="20" t="inlineStr">
         <is>
           <t>Patch flag added</t>
@@ -26796,7 +27145,7 @@
         </is>
       </c>
     </row>
-    <row r="112">
+    <row r="112" ht="25.5" customHeight="1">
       <c r="A112" s="31" t="inlineStr">
         <is>
           <t>Missing workbook row</t>
@@ -26840,7 +27189,7 @@
         </is>
       </c>
     </row>
-    <row r="113">
+    <row r="113" ht="25.5" customHeight="1">
       <c r="A113" s="31" t="inlineStr">
         <is>
           <t>Missing workbook row</t>
@@ -26884,7 +27233,7 @@
         </is>
       </c>
     </row>
-    <row r="114">
+    <row r="114" ht="25.5" customHeight="1">
       <c r="A114" s="31" t="inlineStr">
         <is>
           <t>Missing workbook row</t>
@@ -26928,7 +27277,7 @@
         </is>
       </c>
     </row>
-    <row r="115">
+    <row r="115" ht="25.5" customHeight="1">
       <c r="A115" s="31" t="inlineStr">
         <is>
           <t>Missing workbook row</t>

</xml_diff>